<commit_message>
fix: aguarda inicializacao completa do pgAdmin na verificacao Docker
</commit_message>
<xml_diff>
--- a/documentacao/Template_ATDD.xlsx
+++ b/documentacao/Template_ATDD.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pb" sheetId="1" r:id="R052cffce0b334e75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BDD e Testes - relação" sheetId="2" r:id="Rd701ca87728a43e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pb" sheetId="1" r:id="Rc0245e48402f47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BDD e Testes - relação" sheetId="2" r:id="Ra8223e31b3fd499d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -477,7 +477,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -519,6 +519,11 @@
         <x:fgColor rgb="FFFFFF00"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="14">
     <x:border/>
@@ -645,7 +650,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="73">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -822,6 +827,19 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="21" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1175,7 +1193,7 @@
       <x:c r="A5" s="2">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B5" s="72" t="str">
+      <x:c r="B5" s="75" t="str">
         <x:v>ALUNO BÁSICO
 US e BDD: Gustavo Camargo</x:v>
       </x:c>
@@ -1208,13 +1226,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M5" s="30"/>
-      <x:c r="N5" s="71" t="str">
+      <x:c r="N5" s="76" t="str">
         <x:v>AlunoTest e AlunoControllerTest: 12º curso, limite 7,0, nota insuficiente, curso repetido, evento único.</x:v>
       </x:c>
-      <x:c r="O5" s="71" t="str">
+      <x:c r="O5" s="76" t="str">
         <x:v>Executado em 14/09/2026. JUnit/Maven: 37 testes, nenhuma falha. H2 e PostgreSQL reais.</x:v>
       </x:c>
-      <x:c r="P5" s="71" t="str">
+      <x:c r="P5" s="76" t="str">
         <x:v>Plano PREMIUM no 12º curso válido. Média &lt; 7 não conta. Evento de promoção publicado uma única vez.</x:v>
       </x:c>
       <x:c r="Q5" s="45"/>
@@ -1225,7 +1243,7 @@
       <x:c r="A6" s="2">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="72" t="str">
+      <x:c r="B6" s="75" t="str">
         <x:v>ALUNO PREMIUM
 US e BDD: Gustavo Champam</x:v>
       </x:c>
@@ -1258,13 +1276,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="M6" s="30"/>
-      <x:c r="N6" s="71" t="str">
+      <x:c r="N6" s="76" t="str">
         <x:v>AlunoPremiumTest e RecompensaAceitacaoTest: 1 voucher, 3 moedas, origem registrada e reprocessamento sem duplicação.</x:v>
       </x:c>
-      <x:c r="O6" s="71" t="str">
+      <x:c r="O6" s="76" t="str">
         <x:v>Executado em 14/09/2026. JUnit/Maven: 37 testes, nenhuma falha. JaCoCo: 100% linhas e ramos de todas as classes.</x:v>
       </x:c>
-      <x:c r="P6" s="71" t="str">
+      <x:c r="P6" s="76" t="str">
         <x:v>Carteira habilitada no Premium. Saldo de 1 voucher e 3 moedas. Histórico: PROMOCAO_PREMIUM e data. Um registro por aluno.</x:v>
       </x:c>
       <x:c r="Q6" s="45"/>
@@ -2367,112 +2385,112 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="59" t="str">
+      <x:c r="A1" s="77" t="str">
         <x:v>VISÃO DO PRODUTO: Educação Continuada Gamificada. Incentivar a conclusão de cursos com promoção de plano e recompensas.</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
-      <x:c r="A2" s="59" t="str">
+      <x:c r="A2" s="77" t="str">
         <x:v>FUNCIONALIDADES / USER STORIES</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="38" customHeight="1">
-      <x:c r="A3" s="59" t="str">
+      <x:c r="A3" s="77" t="str">
         <x:v>US01 — Gustavo Camargo: promoção ao Premium após 12 cursos válidos. US02 — Gustavo Champam: receber 1 voucher e 3 moedas com histórico.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="38" customHeight="1">
-      <x:c r="A4" s="59" t="str"/>
+      <x:c r="A4" s="77" t="str"/>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
-      <x:c r="A5" s="59" t="str">
+      <x:c r="A5" s="77" t="str">
         <x:v>Cenários BDD e relação com testes JUnit</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
-      <x:c r="A6" s="59" t="str"/>
+      <x:c r="A6" s="77" t="str"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
-      <x:c r="A7" s="59" t="str">
+      <x:c r="A7" s="77" t="str">
         <x:v>US01 — Gustavo Camargo: promoção no limite de 7,0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
-      <x:c r="A8" s="59" t="str">
+      <x:c r="A8" s="77" t="str">
         <x:v>Dado um aluno Básico com 11 cursos válidos,</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
-      <x:c r="A9" s="59" t="str">
+      <x:c r="A9" s="77" t="str">
         <x:v>Quando conclui um curso distinto com média 7,0,</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
-      <x:c r="A10" s="59" t="str">
+      <x:c r="A10" s="77" t="str">
         <x:v>Então passa ao Premium, totaliza 12 cursos e publica um evento.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
-      <x:c r="A11" s="59" t="str">
+      <x:c r="A11" s="77" t="str">
         <x:v>Testes: AlunoTest e AlunoControllerTest.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
-      <x:c r="A12" s="59" t="str"/>
+      <x:c r="A12" s="77" t="str"/>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
-      <x:c r="A13" s="59" t="str">
+      <x:c r="A13" s="77" t="str">
         <x:v>US01 — Gustavo Camargo: média insuficiente</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
-      <x:c r="A14" s="59" t="str">
+      <x:c r="A14" s="77" t="str">
         <x:v>Dado um aluno Básico com 11 cursos, quando registra média 6,99,</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
-      <x:c r="A15" s="59" t="str">
+      <x:c r="A15" s="77" t="str">
         <x:v>Então permanece Básico com 11 cursos e pode tentar novamente.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
-      <x:c r="A16" s="59" t="str"/>
+      <x:c r="A16" s="77" t="str"/>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
-      <x:c r="A17" s="59" t="str">
+      <x:c r="A17" s="77" t="str">
         <x:v>US02 — Gustavo Champam: prêmios e origem</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
-      <x:c r="A18" s="59" t="str">
+      <x:c r="A18" s="77" t="str">
         <x:v>Dado um aluno promovido, quando o evento é processado,</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
-      <x:c r="A19" s="59" t="str">
+      <x:c r="A19" s="77" t="str">
         <x:v>Então recebe 1 voucher e 3 moedas e o histórico registra PROMOCAO_PREMIUM e data.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
-      <x:c r="A20" s="59" t="str">
+      <x:c r="A20" s="77" t="str">
         <x:v>Testes: AlunoPremiumTest e RecompensaAceitacaoTest.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
-      <x:c r="A21" s="59" t="str"/>
+      <x:c r="A21" s="77" t="str"/>
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
-      <x:c r="A22" s="59" t="str">
+      <x:c r="A22" s="77" t="str">
         <x:v>US02 — Gustavo Champam: reprocessamento</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="38" customHeight="1">
-      <x:c r="A23" s="59" t="str">
+      <x:c r="A23" s="77" t="str">
         <x:v>Quando o evento é recebido novamente ou outro curso é concluído, os prêmios não duplicam.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
-      <x:c r="A24" s="59" t="str">
+      <x:c r="A24" s="77" t="str">
         <x:v>Evidências: evidencias/red, evidencias/green e evidencias/blue. Execução real: 14/09/2026.</x:v>
       </x:c>
     </x:row>

</xml_diff>